<commit_message>
fix(io): fix XLSX date handling with UTC math and add columnFormats metadata
- Fix DST bug in both read/write by using Date.UTC() for timezone-neutral serial number conversion
- Preserve time components in writeXLSX (was stripping to midnight)
- Add datetime format style (yyyy-mm-dd h:mm:ss) for dates with time
- Add columnFormats to readXLSXMetadata exposing numFmt codes from xl/styles.xml
- Export XLSXColumnFormat type
</commit_message>
<xml_diff>
--- a/packages/dataframe/ts/io/fixtures/mixed-types.xlsx
+++ b/packages/dataframe/ts/io/fixtures/mixed-types.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jtmenchaca/tidy-ts/src/dataframe/ts/io/fixtures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jtmenchaca/tidy-ts/packages/dataframe/ts/io/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{18A6CDF6-A8D7-304F-A421-BD815282FA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{214C8FD1-8BAF-304E-909D-103FA748D30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1900" yWindow="1820" windowWidth="27240" windowHeight="16440" xr2:uid="{C7FA88AD-8CF9-AE42-B979-DC0AE0C77448}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>name</t>
   </si>
@@ -45,11 +45,17 @@
   <si>
     <t>Charlie</t>
   </si>
+  <si>
+    <t>datetime</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="m/d/yy\ h:mm;@"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -527,9 +533,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -905,10 +912,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D75B00-D307-EB49-A2E0-4C506F2CC4E6}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="13.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -924,8 +934,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -941,8 +954,11 @@
       <c r="E2" s="1">
         <v>45306</v>
       </c>
+      <c r="F2" s="2">
+        <v>45306.042013888888</v>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -958,8 +974,11 @@
       <c r="E3" s="1">
         <v>45342</v>
       </c>
+      <c r="F3" s="2">
+        <v>45342.166666666664</v>
+      </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -974,6 +993,9 @@
       </c>
       <c r="E4" s="1">
         <v>45361</v>
+      </c>
+      <c r="F4" s="2">
+        <v>45361.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>